<commit_message>
chore: update import template v2 — locked example row and separator
</commit_message>
<xml_diff>
--- a/public/templates/TayoNa_Trip_Import_Template.xlsx
+++ b/public/templates/TayoNa_Trip_Import_Template.xlsx
@@ -56,7 +56,6 @@
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="001F2937"/>
       <sz val="10"/>
     </font>
     <font>
@@ -68,16 +67,17 @@
     <font>
       <name val="Arial"/>
       <i val="1"/>
-      <color rgb="006B7280"/>
+      <color rgb="0092400E"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="006B7280"/>
+      <b val="1"/>
+      <color rgb="00A78BFA"/>
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -116,8 +116,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EDE9FE"/>
-        <bgColor rgb="00EDE9FE"/>
+        <fgColor rgb="00FEF3C7"/>
+        <bgColor rgb="00FEF3C7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F3F0FF"/>
+        <bgColor rgb="00F3F0FF"/>
       </patternFill>
     </fill>
   </fills>
@@ -147,7 +153,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -170,13 +176,20 @@
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+      <protection locked="0" hidden="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -544,7 +557,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -586,7 +599,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Go through each tab (Trip, Destinations, Activities, Members, Budget) and fill in your data.</t>
+          <t>Go through each tab (Trip, Destinations, Activities, Members, Budget) and fill in your data below the separator row.</t>
         </is>
       </c>
     </row>
@@ -610,145 +623,158 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Row 2 in each tab shows an example in purple. You can delete it or leave it — the importer ignores it automatically.</t>
+          <t>Each tab has a yellow ⚠️ EXAMPLE row — it is locked and cannot be edited. Leave it as-is; the importer ignores it automatically.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>4. Dates format</t>
+          <t>4. Separator row</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Use YYYY-MM-DD format for all dates (e.g. 2025-03-15).</t>
+          <t>The dark '▼ Enter your data below this row' is your starting point. Enter data in the rows below it.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>5. Required fields</t>
+          <t>5. Dates format</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Fields marked * are required. Others are optional.</t>
+          <t>Use YYYY-MM-DD format for all dates (e.g. 2025-03-15).</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>6. Save as .xlsx</t>
+          <t>6. Required fields</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Keep the file in Excel format (.xlsx). Google Sheets: File → Download → Microsoft Excel.</t>
+          <t>Fields marked * are required. Others are optional.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>7. Import</t>
+          <t>7. Save as .xlsx</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
+          <t>Keep the file in Excel format (.xlsx). Google Sheets: File → Download → Microsoft Excel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>8. Import</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
           <t>In Tayo Na → Profile → Import Trip → select this file.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="8" customHeight="1"/>
-    <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="3" t="inlineStr">
+    <row r="14" ht="8" customHeight="1"/>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>TABS OVERVIEW</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>Trip</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>Basic trip details — name, dates. One row only.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Destinations</t>
+          <t>Trip</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Each city/place you're visiting. One row per destination.</t>
+          <t>Basic trip details — name, dates. One row only.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Activities</t>
+          <t>Destinations</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Things you want to do. One row per activity.</t>
+          <t>Each city/place you're visiting. One row per destination.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Members</t>
+          <t>Activities</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>People going on the trip. One row per person.</t>
+          <t>Things you want to do. One row per activity.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
         <is>
+          <t>Members</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>People going on the trip. One row per person.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
           <t>Budget</t>
         </is>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B20" s="5" t="inlineStr">
         <is>
           <t>Cost estimates by category. One row per budget item.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="17">
+  <mergeCells count="18">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="B12:F12"/>
     <mergeCell ref="B7:F7"/>
     <mergeCell ref="B6:F6"/>
     <mergeCell ref="B16:F16"/>
-    <mergeCell ref="A14:F14"/>
-    <mergeCell ref="B15:F15"/>
+    <mergeCell ref="B20:F20"/>
     <mergeCell ref="B10:F10"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A5:F5"/>
     <mergeCell ref="B11:F11"/>
+    <mergeCell ref="A15:F15"/>
     <mergeCell ref="B18:F18"/>
     <mergeCell ref="B19:F19"/>
     <mergeCell ref="B8:F8"/>
     <mergeCell ref="A3:F3"/>
     <mergeCell ref="B17:F17"/>
     <mergeCell ref="B9:F9"/>
+    <mergeCell ref="B13:F13"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -761,7 +787,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -810,7 +836,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="9" t="inlineStr">
         <is>
-          <t>Mexico Getaway 2025</t>
+          <t>⚠️ EXAMPLE: Mexico Getaway 2025</t>
         </is>
       </c>
       <c r="B3" s="9" t="inlineStr">
@@ -828,33 +854,47 @@
           <t>Spring break trip!</t>
         </is>
       </c>
-      <c r="E3" s="10" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="11" t="n"/>
-      <c r="B4" s="11" t="n"/>
-      <c r="C4" s="11" t="n"/>
-      <c r="D4" s="11" t="n"/>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>▼  Enter your data below this row</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="5" t="n"/>
-      <c r="B5" s="5" t="n"/>
-      <c r="C5" s="5" t="n"/>
-      <c r="D5" s="5" t="n"/>
+      <c r="A5" s="11" t="n"/>
+      <c r="B5" s="11" t="n"/>
+      <c r="C5" s="11" t="n"/>
+      <c r="D5" s="11" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="11" t="n"/>
-      <c r="B6" s="11" t="n"/>
-      <c r="C6" s="11" t="n"/>
-      <c r="D6" s="11" t="n"/>
+      <c r="A6" s="12" t="n"/>
+      <c r="B6" s="12" t="n"/>
+      <c r="C6" s="12" t="n"/>
+      <c r="D6" s="12" t="n"/>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="11" t="n"/>
+      <c r="B7" s="11" t="n"/>
+      <c r="C7" s="11" t="n"/>
+      <c r="D7" s="11" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="DF99"/>
+  <mergeCells count="2">
     <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A4:D4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -867,7 +907,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -922,7 +962,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="9" t="inlineStr">
         <is>
-          <t>Tulum</t>
+          <t>⚠️ EXAMPLE: Tulum</t>
         </is>
       </c>
       <c r="B3" s="9" t="inlineStr">
@@ -945,71 +985,85 @@
           <t>Beach vibes ☀️</t>
         </is>
       </c>
-      <c r="F3" s="10" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="11" t="n"/>
-      <c r="B4" s="11" t="n"/>
-      <c r="C4" s="11" t="n"/>
-      <c r="D4" s="11" t="n"/>
-      <c r="E4" s="11" t="n"/>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>▼  Enter your data below this row</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="5" t="n"/>
-      <c r="B5" s="5" t="n"/>
-      <c r="C5" s="5" t="n"/>
-      <c r="D5" s="5" t="n"/>
-      <c r="E5" s="5" t="n"/>
+      <c r="A5" s="11" t="n"/>
+      <c r="B5" s="11" t="n"/>
+      <c r="C5" s="11" t="n"/>
+      <c r="D5" s="11" t="n"/>
+      <c r="E5" s="11" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="11" t="n"/>
-      <c r="B6" s="11" t="n"/>
-      <c r="C6" s="11" t="n"/>
-      <c r="D6" s="11" t="n"/>
-      <c r="E6" s="11" t="n"/>
+      <c r="A6" s="12" t="n"/>
+      <c r="B6" s="12" t="n"/>
+      <c r="C6" s="12" t="n"/>
+      <c r="D6" s="12" t="n"/>
+      <c r="E6" s="12" t="n"/>
     </row>
     <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="5" t="n"/>
-      <c r="B7" s="5" t="n"/>
-      <c r="C7" s="5" t="n"/>
-      <c r="D7" s="5" t="n"/>
-      <c r="E7" s="5" t="n"/>
+      <c r="A7" s="11" t="n"/>
+      <c r="B7" s="11" t="n"/>
+      <c r="C7" s="11" t="n"/>
+      <c r="D7" s="11" t="n"/>
+      <c r="E7" s="11" t="n"/>
     </row>
     <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="11" t="n"/>
-      <c r="B8" s="11" t="n"/>
-      <c r="C8" s="11" t="n"/>
-      <c r="D8" s="11" t="n"/>
-      <c r="E8" s="11" t="n"/>
+      <c r="A8" s="12" t="n"/>
+      <c r="B8" s="12" t="n"/>
+      <c r="C8" s="12" t="n"/>
+      <c r="D8" s="12" t="n"/>
+      <c r="E8" s="12" t="n"/>
     </row>
     <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="5" t="n"/>
-      <c r="B9" s="5" t="n"/>
-      <c r="C9" s="5" t="n"/>
-      <c r="D9" s="5" t="n"/>
-      <c r="E9" s="5" t="n"/>
+      <c r="A9" s="11" t="n"/>
+      <c r="B9" s="11" t="n"/>
+      <c r="C9" s="11" t="n"/>
+      <c r="D9" s="11" t="n"/>
+      <c r="E9" s="11" t="n"/>
     </row>
     <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="11" t="n"/>
-      <c r="B10" s="11" t="n"/>
-      <c r="C10" s="11" t="n"/>
-      <c r="D10" s="11" t="n"/>
-      <c r="E10" s="11" t="n"/>
+      <c r="A10" s="12" t="n"/>
+      <c r="B10" s="12" t="n"/>
+      <c r="C10" s="12" t="n"/>
+      <c r="D10" s="12" t="n"/>
+      <c r="E10" s="12" t="n"/>
     </row>
     <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="5" t="n"/>
-      <c r="B11" s="5" t="n"/>
-      <c r="C11" s="5" t="n"/>
-      <c r="D11" s="5" t="n"/>
-      <c r="E11" s="5" t="n"/>
+      <c r="A11" s="11" t="n"/>
+      <c r="B11" s="11" t="n"/>
+      <c r="C11" s="11" t="n"/>
+      <c r="D11" s="11" t="n"/>
+      <c r="E11" s="11" t="n"/>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="12" t="n"/>
+      <c r="B12" s="12" t="n"/>
+      <c r="C12" s="12" t="n"/>
+      <c r="D12" s="12" t="n"/>
+      <c r="E12" s="12" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="DF99"/>
+  <mergeCells count="2">
     <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A4:E4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1022,7 +1076,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1077,7 +1131,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="9" t="inlineStr">
         <is>
-          <t>Cenote swim</t>
+          <t>⚠️ EXAMPLE: Cenote swim</t>
         </is>
       </c>
       <c r="B3" s="9" t="inlineStr">
@@ -1100,99 +1154,113 @@
           <t>25</t>
         </is>
       </c>
-      <c r="F3" s="10" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="11" t="n"/>
-      <c r="B4" s="11" t="n"/>
-      <c r="C4" s="11" t="n"/>
-      <c r="D4" s="11" t="n"/>
-      <c r="E4" s="11" t="n"/>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>▼  Enter your data below this row</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="5" t="n"/>
-      <c r="B5" s="5" t="n"/>
-      <c r="C5" s="5" t="n"/>
-      <c r="D5" s="5" t="n"/>
-      <c r="E5" s="5" t="n"/>
+      <c r="A5" s="11" t="n"/>
+      <c r="B5" s="11" t="n"/>
+      <c r="C5" s="11" t="n"/>
+      <c r="D5" s="11" t="n"/>
+      <c r="E5" s="11" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="11" t="n"/>
-      <c r="B6" s="11" t="n"/>
-      <c r="C6" s="11" t="n"/>
-      <c r="D6" s="11" t="n"/>
-      <c r="E6" s="11" t="n"/>
+      <c r="A6" s="12" t="n"/>
+      <c r="B6" s="12" t="n"/>
+      <c r="C6" s="12" t="n"/>
+      <c r="D6" s="12" t="n"/>
+      <c r="E6" s="12" t="n"/>
     </row>
     <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="5" t="n"/>
-      <c r="B7" s="5" t="n"/>
-      <c r="C7" s="5" t="n"/>
-      <c r="D7" s="5" t="n"/>
-      <c r="E7" s="5" t="n"/>
+      <c r="A7" s="11" t="n"/>
+      <c r="B7" s="11" t="n"/>
+      <c r="C7" s="11" t="n"/>
+      <c r="D7" s="11" t="n"/>
+      <c r="E7" s="11" t="n"/>
     </row>
     <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="11" t="n"/>
-      <c r="B8" s="11" t="n"/>
-      <c r="C8" s="11" t="n"/>
-      <c r="D8" s="11" t="n"/>
-      <c r="E8" s="11" t="n"/>
+      <c r="A8" s="12" t="n"/>
+      <c r="B8" s="12" t="n"/>
+      <c r="C8" s="12" t="n"/>
+      <c r="D8" s="12" t="n"/>
+      <c r="E8" s="12" t="n"/>
     </row>
     <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="5" t="n"/>
-      <c r="B9" s="5" t="n"/>
-      <c r="C9" s="5" t="n"/>
-      <c r="D9" s="5" t="n"/>
-      <c r="E9" s="5" t="n"/>
+      <c r="A9" s="11" t="n"/>
+      <c r="B9" s="11" t="n"/>
+      <c r="C9" s="11" t="n"/>
+      <c r="D9" s="11" t="n"/>
+      <c r="E9" s="11" t="n"/>
     </row>
     <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="11" t="n"/>
-      <c r="B10" s="11" t="n"/>
-      <c r="C10" s="11" t="n"/>
-      <c r="D10" s="11" t="n"/>
-      <c r="E10" s="11" t="n"/>
+      <c r="A10" s="12" t="n"/>
+      <c r="B10" s="12" t="n"/>
+      <c r="C10" s="12" t="n"/>
+      <c r="D10" s="12" t="n"/>
+      <c r="E10" s="12" t="n"/>
     </row>
     <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="5" t="n"/>
-      <c r="B11" s="5" t="n"/>
-      <c r="C11" s="5" t="n"/>
-      <c r="D11" s="5" t="n"/>
-      <c r="E11" s="5" t="n"/>
+      <c r="A11" s="11" t="n"/>
+      <c r="B11" s="11" t="n"/>
+      <c r="C11" s="11" t="n"/>
+      <c r="D11" s="11" t="n"/>
+      <c r="E11" s="11" t="n"/>
     </row>
     <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="11" t="n"/>
-      <c r="B12" s="11" t="n"/>
-      <c r="C12" s="11" t="n"/>
-      <c r="D12" s="11" t="n"/>
-      <c r="E12" s="11" t="n"/>
+      <c r="A12" s="12" t="n"/>
+      <c r="B12" s="12" t="n"/>
+      <c r="C12" s="12" t="n"/>
+      <c r="D12" s="12" t="n"/>
+      <c r="E12" s="12" t="n"/>
     </row>
     <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="5" t="n"/>
-      <c r="B13" s="5" t="n"/>
-      <c r="C13" s="5" t="n"/>
-      <c r="D13" s="5" t="n"/>
-      <c r="E13" s="5" t="n"/>
+      <c r="A13" s="11" t="n"/>
+      <c r="B13" s="11" t="n"/>
+      <c r="C13" s="11" t="n"/>
+      <c r="D13" s="11" t="n"/>
+      <c r="E13" s="11" t="n"/>
     </row>
     <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="11" t="n"/>
-      <c r="B14" s="11" t="n"/>
-      <c r="C14" s="11" t="n"/>
-      <c r="D14" s="11" t="n"/>
-      <c r="E14" s="11" t="n"/>
+      <c r="A14" s="12" t="n"/>
+      <c r="B14" s="12" t="n"/>
+      <c r="C14" s="12" t="n"/>
+      <c r="D14" s="12" t="n"/>
+      <c r="E14" s="12" t="n"/>
     </row>
     <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="5" t="n"/>
-      <c r="B15" s="5" t="n"/>
-      <c r="C15" s="5" t="n"/>
-      <c r="D15" s="5" t="n"/>
-      <c r="E15" s="5" t="n"/>
+      <c r="A15" s="11" t="n"/>
+      <c r="B15" s="11" t="n"/>
+      <c r="C15" s="11" t="n"/>
+      <c r="D15" s="11" t="n"/>
+      <c r="E15" s="11" t="n"/>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="12" t="n"/>
+      <c r="B16" s="12" t="n"/>
+      <c r="C16" s="12" t="n"/>
+      <c r="D16" s="12" t="n"/>
+      <c r="E16" s="12" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="DF99"/>
+  <mergeCells count="2">
     <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A4:E4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1205,7 +1273,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1247,7 +1315,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="9" t="inlineStr">
         <is>
-          <t>Dann</t>
+          <t>⚠️ EXAMPLE: Dann</t>
         </is>
       </c>
       <c r="B3" s="9" t="inlineStr">
@@ -1260,55 +1328,69 @@
           <t>Organizer</t>
         </is>
       </c>
-      <c r="D3" s="10" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="11" t="n"/>
-      <c r="B4" s="11" t="n"/>
-      <c r="C4" s="11" t="n"/>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>▼  Enter your data below this row</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="5" t="n"/>
-      <c r="B5" s="5" t="n"/>
-      <c r="C5" s="5" t="n"/>
+      <c r="A5" s="11" t="n"/>
+      <c r="B5" s="11" t="n"/>
+      <c r="C5" s="11" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="11" t="n"/>
-      <c r="B6" s="11" t="n"/>
-      <c r="C6" s="11" t="n"/>
+      <c r="A6" s="12" t="n"/>
+      <c r="B6" s="12" t="n"/>
+      <c r="C6" s="12" t="n"/>
     </row>
     <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="5" t="n"/>
-      <c r="B7" s="5" t="n"/>
-      <c r="C7" s="5" t="n"/>
+      <c r="A7" s="11" t="n"/>
+      <c r="B7" s="11" t="n"/>
+      <c r="C7" s="11" t="n"/>
     </row>
     <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="11" t="n"/>
-      <c r="B8" s="11" t="n"/>
-      <c r="C8" s="11" t="n"/>
+      <c r="A8" s="12" t="n"/>
+      <c r="B8" s="12" t="n"/>
+      <c r="C8" s="12" t="n"/>
     </row>
     <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="5" t="n"/>
-      <c r="B9" s="5" t="n"/>
-      <c r="C9" s="5" t="n"/>
+      <c r="A9" s="11" t="n"/>
+      <c r="B9" s="11" t="n"/>
+      <c r="C9" s="11" t="n"/>
     </row>
     <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="11" t="n"/>
-      <c r="B10" s="11" t="n"/>
-      <c r="C10" s="11" t="n"/>
+      <c r="A10" s="12" t="n"/>
+      <c r="B10" s="12" t="n"/>
+      <c r="C10" s="12" t="n"/>
     </row>
     <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="5" t="n"/>
-      <c r="B11" s="5" t="n"/>
-      <c r="C11" s="5" t="n"/>
+      <c r="A11" s="11" t="n"/>
+      <c r="B11" s="11" t="n"/>
+      <c r="C11" s="11" t="n"/>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="12" t="n"/>
+      <c r="B12" s="12" t="n"/>
+      <c r="C12" s="12" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="DF99"/>
+  <mergeCells count="2">
     <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A4:C4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1321,7 +1403,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1377,7 +1459,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="9" t="inlineStr">
         <is>
-          <t>Flights</t>
+          <t>⚠️ EXAMPLE: Flights</t>
         </is>
       </c>
       <c r="B3" s="9" t="inlineStr">
@@ -1396,85 +1478,99 @@
           <t>Book by Jan</t>
         </is>
       </c>
-      <c r="F3" s="10" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="11" t="n"/>
-      <c r="B4" s="11" t="n"/>
-      <c r="C4" s="11" t="n"/>
-      <c r="D4" s="11" t="n"/>
-      <c r="E4" s="11" t="n"/>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>▼  Enter your data below this row</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="5" t="n"/>
-      <c r="B5" s="5" t="n"/>
-      <c r="C5" s="5" t="n"/>
-      <c r="D5" s="5" t="n"/>
-      <c r="E5" s="5" t="n"/>
+      <c r="A5" s="11" t="n"/>
+      <c r="B5" s="11" t="n"/>
+      <c r="C5" s="11" t="n"/>
+      <c r="D5" s="11" t="n"/>
+      <c r="E5" s="11" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="11" t="n"/>
-      <c r="B6" s="11" t="n"/>
-      <c r="C6" s="11" t="n"/>
-      <c r="D6" s="11" t="n"/>
-      <c r="E6" s="11" t="n"/>
+      <c r="A6" s="12" t="n"/>
+      <c r="B6" s="12" t="n"/>
+      <c r="C6" s="12" t="n"/>
+      <c r="D6" s="12" t="n"/>
+      <c r="E6" s="12" t="n"/>
     </row>
     <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="5" t="n"/>
-      <c r="B7" s="5" t="n"/>
-      <c r="C7" s="5" t="n"/>
-      <c r="D7" s="5" t="n"/>
-      <c r="E7" s="5" t="n"/>
+      <c r="A7" s="11" t="n"/>
+      <c r="B7" s="11" t="n"/>
+      <c r="C7" s="11" t="n"/>
+      <c r="D7" s="11" t="n"/>
+      <c r="E7" s="11" t="n"/>
     </row>
     <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="11" t="n"/>
-      <c r="B8" s="11" t="n"/>
-      <c r="C8" s="11" t="n"/>
-      <c r="D8" s="11" t="n"/>
-      <c r="E8" s="11" t="n"/>
+      <c r="A8" s="12" t="n"/>
+      <c r="B8" s="12" t="n"/>
+      <c r="C8" s="12" t="n"/>
+      <c r="D8" s="12" t="n"/>
+      <c r="E8" s="12" t="n"/>
     </row>
     <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="5" t="n"/>
-      <c r="B9" s="5" t="n"/>
-      <c r="C9" s="5" t="n"/>
-      <c r="D9" s="5" t="n"/>
-      <c r="E9" s="5" t="n"/>
+      <c r="A9" s="11" t="n"/>
+      <c r="B9" s="11" t="n"/>
+      <c r="C9" s="11" t="n"/>
+      <c r="D9" s="11" t="n"/>
+      <c r="E9" s="11" t="n"/>
     </row>
     <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="11" t="n"/>
-      <c r="B10" s="11" t="n"/>
-      <c r="C10" s="11" t="n"/>
-      <c r="D10" s="11" t="n"/>
-      <c r="E10" s="11" t="n"/>
+      <c r="A10" s="12" t="n"/>
+      <c r="B10" s="12" t="n"/>
+      <c r="C10" s="12" t="n"/>
+      <c r="D10" s="12" t="n"/>
+      <c r="E10" s="12" t="n"/>
     </row>
     <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="5" t="n"/>
-      <c r="B11" s="5" t="n"/>
-      <c r="C11" s="5" t="n"/>
-      <c r="D11" s="5" t="n"/>
-      <c r="E11" s="5" t="n"/>
+      <c r="A11" s="11" t="n"/>
+      <c r="B11" s="11" t="n"/>
+      <c r="C11" s="11" t="n"/>
+      <c r="D11" s="11" t="n"/>
+      <c r="E11" s="11" t="n"/>
     </row>
     <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="11" t="n"/>
-      <c r="B12" s="11" t="n"/>
-      <c r="C12" s="11" t="n"/>
-      <c r="D12" s="11" t="n"/>
-      <c r="E12" s="11" t="n"/>
+      <c r="A12" s="12" t="n"/>
+      <c r="B12" s="12" t="n"/>
+      <c r="C12" s="12" t="n"/>
+      <c r="D12" s="12" t="n"/>
+      <c r="E12" s="12" t="n"/>
     </row>
     <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="5" t="n"/>
-      <c r="B13" s="5" t="n"/>
-      <c r="C13" s="5" t="n"/>
-      <c r="D13" s="5" t="n"/>
-      <c r="E13" s="5" t="n"/>
+      <c r="A13" s="11" t="n"/>
+      <c r="B13" s="11" t="n"/>
+      <c r="C13" s="11" t="n"/>
+      <c r="D13" s="11" t="n"/>
+      <c r="E13" s="11" t="n"/>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="12" t="n"/>
+      <c r="B14" s="12" t="n"/>
+      <c r="C14" s="12" t="n"/>
+      <c r="D14" s="12" t="n"/>
+      <c r="E14" s="12" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="DF99"/>
+  <mergeCells count="2">
     <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A4:E4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>